<commit_message>
Configure Vercel deployment and Google Sheets sync
</commit_message>
<xml_diff>
--- a/staff_presence.xlsx
+++ b/staff_presence.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -552,6 +552,295 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>STAFF074</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>19:16:32</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>STAFF895</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>20:56:29</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>STAFF570</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>21:04:01</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>STAFF649</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>12:31:26</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>A / Admin Block</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>STAFF543</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>13:34:21</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>STAFF648</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>13:51:54</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>STAFF674</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>15:45:50</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Steve Jobs</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>STAFF407</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>15:47:33</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Steve Jobs</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>STAFF963</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>15:55:05</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Steve Jobs</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>STAFF180</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>09:46:51</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>C-Block</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>STAFF813</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>12:13:15</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Invisible Statue</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>STAFF907</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>12:16:37</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Steve Jobs</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>STAFF712</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>12:18:48</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Steve Jobs</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>STAFF695</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>12:56:36</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>STAFF567</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13:59:07</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>STAFF193</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>14:24:25</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>STAFF045</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>22:05:33</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>A / Admin Block</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove admin login requirements and sync punches directly to Google Sheets
</commit_message>
<xml_diff>
--- a/staff_presence.xlsx
+++ b/staff_presence.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -841,6 +841,23 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>STAFF001</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>22:47:26</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Connect to user's new Google Sheets webhook
</commit_message>
<xml_diff>
--- a/staff_presence.xlsx
+++ b/staff_presence.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -858,6 +858,23 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>STAFF002</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>23:06:23</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>A / Admin Block</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Enforce once-per-day punch restriction in Indian Standard Time (IST)
</commit_message>
<xml_diff>
--- a/staff_presence.xlsx
+++ b/staff_presence.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -875,6 +875,40 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>STAFF010</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>23:11:27</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>A / Admin Block</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>STAFF020</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>23:12:27</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>A / Admin Block</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Date column to attendance tracker and Google Sheets integration
</commit_message>
<xml_diff>
--- a/staff_presence.xlsx
+++ b/staff_presence.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -909,6 +909,28 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>STAFF030</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>23:15:39</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>A / Admin Block</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>